<commit_message>
📊 [auto] Economic data update — 2026-08-13 14:16 UTC
</commit_message>
<xml_diff>
--- a/reports/excel/MacroPulse_2026-08-13.xlsx
+++ b/reports/excel/MacroPulse_2026-08-13.xlsx
@@ -651,7 +651,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>
@@ -988,12 +988,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>286.8</t>
+          <t>284.1</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>8.27%</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-0.78%</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>5.51%</t>
+          <t>4.66%</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>-0.28%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🔥 通膨指標　歷史數據　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>🔥 通膨指標　歷史數據　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>
@@ -14227,17 +14227,17 @@
       </c>
       <c r="N119" s="20" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>276.1</t>
         </is>
       </c>
       <c r="O119" s="6" t="inlineStr">
         <is>
-          <t>6.78%</t>
+          <t>6.80%</t>
         </is>
       </c>
       <c r="P119" s="20" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="Q119" s="20" t="inlineStr">
@@ -14247,7 +14247,7 @@
       </c>
       <c r="R119" s="6" t="inlineStr">
         <is>
-          <t>4.29%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="S119" s="20" t="inlineStr">
@@ -14329,27 +14329,27 @@
       </c>
       <c r="O120" s="6" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="P120" s="19" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="Q120" s="19" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>156.1</t>
         </is>
       </c>
       <c r="R120" s="6" t="inlineStr">
         <is>
-          <t>5.67%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="S120" s="19" t="inlineStr">
         <is>
-          <t>1.05%</t>
+          <t>1.09%</t>
         </is>
       </c>
     </row>
@@ -14426,27 +14426,27 @@
       </c>
       <c r="O121" s="6" t="inlineStr">
         <is>
-          <t>12.30%</t>
+          <t>12.31%</t>
         </is>
       </c>
       <c r="P121" s="20" t="inlineStr">
         <is>
-          <t>2.73%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="Q121" s="20" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>156.8</t>
         </is>
       </c>
       <c r="R121" s="6" t="inlineStr">
         <is>
-          <t>5.97%</t>
+          <t>5.83%</t>
         </is>
       </c>
       <c r="S121" s="20" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>0.45%</t>
         </is>
       </c>
     </row>
@@ -14518,17 +14518,17 @@
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>286.8</t>
+          <t>286.3</t>
         </is>
       </c>
       <c r="O122" s="6" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="P122" s="19" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-1.46%</t>
         </is>
       </c>
       <c r="Q122" s="19" t="inlineStr">
@@ -14538,12 +14538,12 @@
       </c>
       <c r="R122" s="6" t="inlineStr">
         <is>
-          <t>5.51%</t>
+          <t>5.54%</t>
         </is>
       </c>
       <c r="S122" s="19" t="inlineStr">
         <is>
-          <t>-0.28%</t>
+          <t>-0.11%</t>
         </is>
       </c>
     </row>
@@ -14615,32 +14615,32 @@
       </c>
       <c r="N123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O123" s="20" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>284.1</t>
+        </is>
+      </c>
+      <c r="O123" s="6" t="inlineStr">
+        <is>
+          <t>8.27%</t>
         </is>
       </c>
       <c r="P123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-0.78%</t>
         </is>
       </c>
       <c r="Q123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R123" s="20" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>156.6</t>
+        </is>
+      </c>
+      <c r="R123" s="6" t="inlineStr">
+        <is>
+          <t>4.66%</t>
         </is>
       </c>
       <c r="S123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-0.03%</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14688,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>📈 經濟成長　歷史數據　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>📈 經濟成長　歷史數據　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>👷 勞動市場　歷史數據　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>👷 勞動市場　歷史數據　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>
@@ -36517,7 +36517,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏦 利率與債券　歷史數據　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>🏦 利率與債券　歷史數據　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>
@@ -48336,7 +48336,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>💭 信心指數　歷史數據　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>💭 信心指數　歷史數據　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>
@@ -56513,7 +56513,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>
@@ -59729,7 +59729,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏠 房市　歷史數據　　生成時間：2026-08-13 13:55 UTC</t>
+          <t>🏠 房市　歷史數據　　生成時間：2026-08-13 14:16 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>